<commit_message>
forgot to ever push the milestone document ;(
</commit_message>
<xml_diff>
--- a/Milestones.xlsx
+++ b/Milestones.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/23ad17d4e78749bf/Dokumente/UNILU/FS25/DataMining/voting_prediction/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7F0420DC-F4EB-49C9-9B67-6880824DC34C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="29" documentId="8_{7F0420DC-F4EB-49C9-9B67-6880824DC34C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7B347725-25AA-44F8-AC61-CB8D8CE8C6C8}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5E91E219-AFCD-4E20-B940-506A8E4FC49E}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="26">
   <si>
     <t>What</t>
   </si>
@@ -69,6 +69,51 @@
   </si>
   <si>
     <t xml:space="preserve">Try to find as many useful open Text answers as possible. </t>
+  </si>
+  <si>
+    <t>45'</t>
+  </si>
+  <si>
+    <t>Set up connection to Chat gpt</t>
+  </si>
+  <si>
+    <t>Set up prompt</t>
+  </si>
+  <si>
+    <t>Select cases</t>
+  </si>
+  <si>
+    <t>60'</t>
+  </si>
+  <si>
+    <t>include error message, when chat gpt does not answer.</t>
+  </si>
+  <si>
+    <t>Build test loop</t>
+  </si>
+  <si>
+    <t>Make data cleaning script</t>
+  </si>
+  <si>
+    <t>Build text only loop using 1000 cases</t>
+  </si>
+  <si>
+    <t>Build numeric only loop using 1000 cases</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Make Logistic Regression </t>
+  </si>
+  <si>
+    <t>Analyze results</t>
+  </si>
+  <si>
+    <t>Make a combined model</t>
+  </si>
+  <si>
+    <t>as long as needed</t>
+  </si>
+  <si>
+    <t>Write report, document stuff, etc.</t>
   </si>
 </sst>
 </file>
@@ -500,60 +545,135 @@
       <c r="A5">
         <v>4</v>
       </c>
+      <c r="B5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
+      <c r="B7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
+      <c r="B8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
+      <c r="B9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
+      <c r="B10" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
+      <c r="B11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
+      <c r="B12" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
+      <c r="B13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
+      <c r="B14" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
+      <c r="B15" t="s">
+        <v>6</v>
+      </c>
+      <c r="C15" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>24</v>
+      </c>
+      <c r="C16" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>